<commit_message>
further update to the geometric report, added a new test file, and updated the dynamo script for the geometric evaluator.
</commit_message>
<xml_diff>
--- a/N2_Master_Geometric_Report.xlsx
+++ b/N2_Master_Geometric_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ingeropgroup-my.sharepoint.com/personal/kymaharaj_ingerop_co_za/Documents/Desktop/Python_Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_22E3EDF2068C97BC066AAE56385BDA16E6C0FB9C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4543EB89-FCBA-4DE9-AFA6-0DD577C3A085}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_6AAB0EF437249F9CCA8AB556385BDA16E6C0DB31" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF34649B-EB31-4515-8A4C-CC91C89F52C8}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2124" yWindow="1020" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vertical Checks" sheetId="1" r:id="rId1"/>
@@ -128,6 +128,9 @@
     <t>191.08</t>
   </si>
   <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
     <t>19.999, 19.999, 19.999, 19.999, 19.999, 19.999, 19.999, 19.999, 19.999, 11.075</t>
   </si>
   <si>
@@ -195,9 +198,6 @@
   </si>
   <si>
     <t>9.33</t>
-  </si>
-  <si>
-    <t>CRITICAL</t>
   </si>
   <si>
     <t>9.335</t>
@@ -1041,7 +1041,7 @@
         <v>13</v>
       </c>
       <c r="L2" s="2">
-        <v>202.08</v>
+        <v>280.95999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -1079,7 +1079,7 @@
         <v>13</v>
       </c>
       <c r="L3" s="2">
-        <v>201.34</v>
+        <v>279.82</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1117,7 +1117,7 @@
         <v>13</v>
       </c>
       <c r="L4" s="2">
-        <v>181.3</v>
+        <v>249.1</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1155,7 +1155,7 @@
         <v>52.356999999999999</v>
       </c>
       <c r="L5" s="2">
-        <v>197.47</v>
+        <v>273.87</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -1193,7 +1193,7 @@
         <v>41.21</v>
       </c>
       <c r="L6" s="2">
-        <v>230.5</v>
+        <v>325.13</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1231,7 +1231,7 @@
         <v>13</v>
       </c>
       <c r="L7" s="2">
-        <v>198.85</v>
+        <v>275.99</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -1269,7 +1269,7 @@
         <v>13</v>
       </c>
       <c r="L8" s="2">
-        <v>198.4</v>
+        <v>275.3</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -1307,7 +1307,7 @@
         <v>13</v>
       </c>
       <c r="L9" s="2">
-        <v>199.15</v>
+        <v>276.45</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="L10" s="2">
-        <v>201.38</v>
+        <v>279.89</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -1383,7 +1383,7 @@
         <v>13</v>
       </c>
       <c r="L11" s="2">
-        <v>201.99</v>
+        <v>280.82</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -1421,7 +1421,7 @@
         <v>13</v>
       </c>
       <c r="L12" s="2">
-        <v>200.7</v>
+        <v>278.83999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -1459,7 +1459,7 @@
         <v>13</v>
       </c>
       <c r="L13" s="2">
-        <v>201.35</v>
+        <v>279.85000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -1497,7 +1497,7 @@
         <v>13</v>
       </c>
       <c r="L14" s="2">
-        <v>184.08</v>
+        <v>253.35</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -1535,7 +1535,7 @@
         <v>87.549000000000007</v>
       </c>
       <c r="L15" s="2">
-        <v>200.95</v>
+        <v>279.22000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -1573,7 +1573,7 @@
         <v>13</v>
       </c>
       <c r="L16" s="2">
-        <v>211.11</v>
+        <v>294.93</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
@@ -1611,7 +1611,7 @@
         <v>80.793000000000006</v>
       </c>
       <c r="L17" s="2">
-        <v>220.91</v>
+        <v>310.14999999999998</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
@@ -1649,7 +1649,7 @@
         <v>13</v>
       </c>
       <c r="L18" s="2">
-        <v>186</v>
+        <v>256.27999999999997</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
@@ -1687,7 +1687,7 @@
         <v>96.903999999999996</v>
       </c>
       <c r="L19" s="2">
-        <v>196.3</v>
+        <v>272.06</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
@@ -1725,7 +1725,7 @@
         <v>96.682000000000002</v>
       </c>
       <c r="L20" s="2">
-        <v>207.2</v>
+        <v>288.88</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
@@ -1763,7 +1763,7 @@
         <v>13</v>
       </c>
       <c r="L21" s="2">
-        <v>189.16</v>
+        <v>261.11</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
@@ -1801,7 +1801,7 @@
         <v>106.336</v>
       </c>
       <c r="L22" s="2">
-        <v>200.12</v>
+        <v>277.94</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -1839,7 +1839,7 @@
         <v>99.322999999999993</v>
       </c>
       <c r="L23" s="2">
-        <v>224.96</v>
+        <v>316.47000000000003</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
@@ -1877,7 +1877,7 @@
         <v>102.43600000000001</v>
       </c>
       <c r="L24" s="2">
-        <v>195.18</v>
+        <v>270.35000000000002</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
@@ -1915,7 +1915,7 @@
         <v>13</v>
       </c>
       <c r="L25" s="2">
-        <v>232.28</v>
+        <v>327.92</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
@@ -1953,7 +1953,7 @@
         <v>13</v>
       </c>
       <c r="L26" s="2">
-        <v>231.27</v>
+        <v>326.33</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
@@ -1991,7 +1991,7 @@
         <v>13</v>
       </c>
       <c r="L27" s="2">
-        <v>213.09</v>
+        <v>297.99</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
@@ -2029,7 +2029,7 @@
         <v>13</v>
       </c>
       <c r="L28" s="2">
-        <v>231.62</v>
+        <v>326.87</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
@@ -2067,7 +2067,7 @@
         <v>13</v>
       </c>
       <c r="L29" s="2">
-        <v>206.95</v>
+        <v>288.49</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
@@ -2105,7 +2105,7 @@
         <v>13</v>
       </c>
       <c r="L30" s="2">
-        <v>245.66</v>
+        <v>348.94</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
@@ -2143,7 +2143,7 @@
         <v>13</v>
       </c>
       <c r="L31" s="2">
-        <v>205.84</v>
+        <v>286.77</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -2181,7 +2181,7 @@
         <v>15</v>
       </c>
       <c r="L32" s="2">
-        <v>205.29</v>
+        <v>285.92</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -2219,7 +2219,7 @@
         <v>15</v>
       </c>
       <c r="L33" s="2">
-        <v>205.19</v>
+        <v>285.77</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -2257,7 +2257,7 @@
         <v>4.2709999999999999</v>
       </c>
       <c r="L34" s="2">
-        <v>204.99</v>
+        <v>285.45</v>
       </c>
     </row>
   </sheetData>
@@ -2313,7 +2313,7 @@
         <v>25</v>
       </c>
       <c r="D2" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E2" s="2">
         <v>0</v>
@@ -2336,10 +2336,10 @@
         <v>30</v>
       </c>
       <c r="D3" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E3" s="2">
-        <v>0</v>
+        <v>0.87</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>26</v>
@@ -2359,30 +2359,30 @@
         <v>34</v>
       </c>
       <c r="D4" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E4" s="2">
-        <v>1.44</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E5" s="2">
         <v>0</v>
@@ -2391,21 +2391,21 @@
         <v>26</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E6" s="2">
         <v>0</v>
@@ -2414,96 +2414,96 @@
         <v>26</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E7" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E8" s="2">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>26</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E9" s="2">
-        <v>0</v>
+        <v>0.34</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>26</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D10" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E10" s="2">
         <v>6</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>59</v>
@@ -2520,7 +2520,7 @@
         <v>62</v>
       </c>
       <c r="D11" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E11" s="2">
         <v>0</v>
@@ -2543,7 +2543,7 @@
         <v>66</v>
       </c>
       <c r="D12" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
@@ -2566,13 +2566,13 @@
         <v>69</v>
       </c>
       <c r="D13" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>70</v>
@@ -2589,7 +2589,7 @@
         <v>73</v>
       </c>
       <c r="D14" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E14" s="2">
         <v>0</v>
@@ -2612,7 +2612,7 @@
         <v>76</v>
       </c>
       <c r="D15" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E15" s="2">
         <v>0</v>
@@ -2635,7 +2635,7 @@
         <v>79</v>
       </c>
       <c r="D16" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E16" s="2">
         <v>0</v>
@@ -2658,7 +2658,7 @@
         <v>82</v>
       </c>
       <c r="D17" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E17" s="2">
         <v>0</v>
@@ -2675,16 +2675,16 @@
         <v>84</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E18" s="2">
-        <v>0</v>
+        <v>0.34</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>26</v>
@@ -2704,7 +2704,7 @@
         <v>88</v>
       </c>
       <c r="D19" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E19" s="2">
         <v>0</v>
@@ -2727,7 +2727,7 @@
         <v>91</v>
       </c>
       <c r="D20" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E20" s="2">
         <v>0</v>
@@ -2750,7 +2750,7 @@
         <v>95</v>
       </c>
       <c r="D21" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E21" s="2">
         <v>0</v>
@@ -2767,16 +2767,16 @@
         <v>97</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>98</v>
       </c>
       <c r="D22" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E22" s="2">
-        <v>0</v>
+        <v>0.34</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>26</v>
@@ -2790,16 +2790,16 @@
         <v>100</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>101</v>
       </c>
       <c r="D23" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E23" s="2">
-        <v>0</v>
+        <v>0.34</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>26</v>
@@ -2813,16 +2813,16 @@
         <v>103</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D24" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E24" s="2">
-        <v>0</v>
+        <v>0.34</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>26</v>
@@ -2842,7 +2842,7 @@
         <v>107</v>
       </c>
       <c r="D25" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E25" s="2">
         <v>0</v>
@@ -2865,7 +2865,7 @@
         <v>110</v>
       </c>
       <c r="D26" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
@@ -2888,7 +2888,7 @@
         <v>113</v>
       </c>
       <c r="D27" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E27" s="2">
         <v>0</v>
@@ -2911,7 +2911,7 @@
         <v>116</v>
       </c>
       <c r="D28" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E28" s="2">
         <v>0</v>
@@ -2934,10 +2934,10 @@
         <v>120</v>
       </c>
       <c r="D29" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E29" s="2">
-        <v>0</v>
+        <v>1.04</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>26</v>
@@ -2957,13 +2957,13 @@
         <v>124</v>
       </c>
       <c r="D30" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E30" s="2">
-        <v>0</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>125</v>
@@ -2980,10 +2980,10 @@
         <v>128</v>
       </c>
       <c r="D31" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E31" s="2">
-        <v>0</v>
+        <v>5.67</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>26</v>
@@ -3003,7 +3003,7 @@
         <v>131</v>
       </c>
       <c r="D32" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -3026,13 +3026,13 @@
         <v>135</v>
       </c>
       <c r="D33" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E33" s="2">
-        <v>3.12</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>136</v>
@@ -3049,7 +3049,7 @@
         <v>138</v>
       </c>
       <c r="D34" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E34" s="2">
         <v>0</v>
@@ -3072,13 +3072,13 @@
         <v>142</v>
       </c>
       <c r="D35" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E35" s="2">
-        <v>0</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>143</v>
@@ -3095,13 +3095,13 @@
         <v>146</v>
       </c>
       <c r="D36" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E36" s="2">
         <v>6</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>147</v>
@@ -3118,10 +3118,10 @@
         <v>150</v>
       </c>
       <c r="D37" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E37" s="2">
-        <v>0</v>
+        <v>2.34</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>26</v>
@@ -3141,7 +3141,7 @@
         <v>154</v>
       </c>
       <c r="D38" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E38" s="2">
         <v>0</v>
@@ -3164,7 +3164,7 @@
         <v>158</v>
       </c>
       <c r="D39" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E39" s="2">
         <v>0</v>
@@ -3187,7 +3187,7 @@
         <v>161</v>
       </c>
       <c r="D40" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E40" s="2">
         <v>0</v>
@@ -3210,7 +3210,7 @@
         <v>164</v>
       </c>
       <c r="D41" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E41" s="2">
         <v>0</v>
@@ -3233,7 +3233,7 @@
         <v>167</v>
       </c>
       <c r="D42" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E42" s="2">
         <v>0</v>
@@ -3250,13 +3250,13 @@
         <v>169</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>170</v>
       </c>
       <c r="D43" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E43" s="2">
         <v>0</v>
@@ -3279,7 +3279,7 @@
         <v>173</v>
       </c>
       <c r="D44" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E44" s="2">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         <v>176</v>
       </c>
       <c r="D45" s="2">
-        <v>393.7</v>
+        <v>666.98</v>
       </c>
       <c r="E45" s="2">
         <v>0</v>

</xml_diff>